<commit_message>
Commit of 25th March - Assert in LoginTest
</commit_message>
<xml_diff>
--- a/GroceryApplicationProject/src/test/resources/TestData.xlsx
+++ b/GroceryApplicationProject/src/test/resources/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\git\AutomationCourse\GroceryApplicationProject\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ED86CD3-02CC-4AFF-88C3-34F06CF18B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27F696C2-A7CB-4FB9-B8A0-FD7B03F6B24C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginPage" sheetId="1" r:id="rId1"/>
@@ -27,14 +27,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t>qwertyuiop</t>
   </si>
   <si>
-    <t>Arya</t>
-  </si>
-  <si>
     <t>admin</t>
   </si>
   <si>
@@ -57,6 +54,12 @@
   </si>
   <si>
     <t>Go Goa Gone</t>
+  </si>
+  <si>
+    <t>jdghglghn</t>
+  </si>
+  <si>
+    <t>gkdfjhgflkjghd</t>
   </si>
 </sst>
 </file>
@@ -382,15 +385,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
@@ -398,15 +401,15 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
         <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
         <v>0</v>
@@ -429,26 +432,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
         <v>3</v>
-      </c>
-      <c r="B1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
         <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -463,7 +466,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>